<commit_message>
fix(import): NocoBase Excel headers (ID, code, Целое число, ...)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/import/products-nocobase.xlsx
+++ b/import/products-nocobase.xlsx
@@ -419,49 +419,44 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Целое число</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>productType</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>grantDays</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>productType</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>sortOrder</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>active</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>serverId</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>vpn_30</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>30 дней</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -472,22 +467,22 @@
           <t>vpn_extend</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>30 дней</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>10</v>
       </c>
-      <c r="F2" t="b">
+      <c r="G2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>vpn_90</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>90 дней</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -498,22 +493,22 @@
           <t>vpn_extend</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>90 дней</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>20</v>
       </c>
-      <c r="F3" t="b">
+      <c r="G3" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>vpn_180</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>180 дней</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -524,10 +519,15 @@
           <t>vpn_extend</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>180 дней</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>30</v>
       </c>
-      <c r="F4" t="b">
+      <c r="G4" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(import): explain NocoBase duplicates + add serverId column to export
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/import/products-nocobase.xlsx
+++ b/import/products-nocobase.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,11 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>active</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>serverId</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(pricing): remove duplicate labels and force canonical invoice amounts
Use canonical weekly pricing for invoice calculation regardless of stale env price maps, normalize VPN tile titles to avoid dual prices, and refresh import artifacts with updated tariff names.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/import/products-nocobase.xlsx
+++ b/import/products-nocobase.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,11 +461,11 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>vpn_30</t>
+          <t>vpn_7</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -474,11 +474,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>30 дней</t>
+          <t>7 дней · 25 ₽</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
@@ -487,11 +487,11 @@
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>vpn_90</t>
+          <t>vpn_30</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -500,11 +500,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>90 дней</t>
+          <t>30 дней · 100 ₽</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -513,26 +513,104 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
+          <t>vpn_90</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>90</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>vpn_extend</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>90 дней · 300 ₽</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
           <t>vpn_180</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C5" t="n">
         <v>180</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>vpn_extend</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>180 дней</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>180 дней · 600 ₽</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>30</v>
       </c>
-      <c r="G4" t="b">
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>proxy_nl1_7</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>proxy_access</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Proxy NL · 7 дней · 18 ₽</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>proxy_nl1_30</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>proxy_access</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Proxy NL · 30 дней · 72 ₽</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>110</v>
+      </c>
+      <c r="G7" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>